<commit_message>
Update ML models and add revenue prediction
</commit_message>
<xml_diff>
--- a/ML/customer_segmentation/results/cluster_summary.xlsx
+++ b/ML/customer_segmentation/results/cluster_summary.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,39 +429,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cluster</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Purchase_Frequency</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Average_Order_Value</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Total_Orders</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total_Spent</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Days_Since_Last_Purchase</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -469,7 +481,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -489,7 +501,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -509,7 +521,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">

</xml_diff>